<commit_message>
Dashboard update: 2026-04-14 — PICO initial data
</commit_message>
<xml_diff>
--- a/public/PICO_8_MASTER_OUTPUT.xlsx
+++ b/public/PICO_8_MASTER_OUTPUT.xlsx
@@ -854,9 +854,9 @@
 const DATA = {
   period: "Current Period",
   email: {
-    totalSends: 21,
-    avgOpenRate: 0.5371,
-    avgClickRate: 0.0301,
+    totalSends: 0,
+    avgOpenRate: 0,
+    avgClickRate: 0,
     listSize180DO: 0,
   },
   finances: {

</xml_diff>